<commit_message>
Add função para gerar termo de devolução
</commit_message>
<xml_diff>
--- a/relatorio_emprestimos_abertos.xlsx
+++ b/relatorio_emprestimos_abertos.xlsx
@@ -510,7 +510,7 @@
         <v>46259</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>12345</v>
@@ -549,7 +549,7 @@
         <v>46259</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>12345678</v>

</xml_diff>